<commit_message>
RF06a: projeta cotação real e VWAP no front office
</commit_message>
<xml_diff>
--- a/frontend/runner/exemplos/validacao.xlsx
+++ b/frontend/runner/exemplos/validacao.xlsx
@@ -186,13 +186,13 @@
     <t>{"cache-control":"no-store"}</t>
   </si>
   <si>
-    <t>{"/precoBaseTunel":"10.00","/origemBase":"REFERENCIA"}</t>
+    <t>{"/precoBaseTunel":"10.00","/origemBase":"ULTIMO"}</t>
   </si>
   <si>
     <t>{}</t>
   </si>
   <si>
-    <t>{"/codigo":"PRECO_FORA_DO_TUNEL","/detalhes/minimo":"9.00","/detalhes/maximo":"11.00","/detalhes/origemBase":"REFERENCIA"}</t>
+    <t>{"/codigo":"PRECO_FORA_DO_TUNEL","/detalhes/minimo":"9.00","/detalhes/maximo":"11.00","/detalhes/origemBase":"ULTIMO"}</t>
   </si>
   <si>
     <t>{"/codigo":"PRECO_FORA_DO_TUNEL"}</t>
@@ -201,7 +201,7 @@
     <t>{"/codigo":"STOP_LIMIT_INCOERENTE"}</t>
   </si>
   <si>
-    <t>{"/estado":"RECEBIDA","/origemBase":"REFERENCIA"}</t>
+    <t>{"/estado":"RECEBIDA","/origemBase":"ULTIMO"}</t>
   </si>
   <si>
     <t>{"/codigo":"QUANTIDADE_FORA_DO_LOTE","/detalhes/lote":"100"}</t>

</xml_diff>